<commit_message>
Registra Pátio Gourmet e Mari Mari como ex-clientes no inventário oficial e no CLAUDE.md
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNtRG1wGaTmzdzTc1r8f3Q
</commit_message>
<xml_diff>
--- a/docs/nekt/inventario-contas-1743-2026-10-16.xlsx
+++ b/docs/nekt/inventario-contas-1743-2026-10-16.xlsx
@@ -545,6 +545,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -578,7 +579,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Não precisa manter (a validar)</t>
+          <t>Não precisa manter (ex-cliente / duplicata)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -600,7 +601,7 @@
         <v>18</v>
       </c>
       <c r="D5" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -609,7 +610,7 @@
         <v>8</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H5" t="n">
         <v>111</v>
@@ -625,7 +626,7 @@
         <v>41</v>
       </c>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
         <v>3</v>
@@ -637,7 +638,7 @@
         <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H6" t="n">
         <v>61</v>
@@ -687,13 +688,13 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
         <v>4</v>
@@ -743,13 +744,13 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" t="n">
         <v>1</v>
@@ -771,13 +772,13 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" t="n">
         <v>1</v>
@@ -818,6 +819,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
@@ -828,14 +830,14 @@
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>• Meta Ads: 71 contas com fonte publicada e execução com sucesso (7 antigas + 64 novas publicadas em 14/10; 7 delas sem veiculação, 0 linhas de insight; 2 de contas desabilitadas na Meta, só histórico). 14 bloqueadas: 12 por 403 ads_read (a conta não está atribuída ao usuário que autorizou), 1 por erro 400 no stream ads e 1 arquivada em 03/09. 18 rascunhos aguardam OAuth. Conectada não significa dado na Trusted: as novas só entram depois da execução agendada de terça 20/10.</t>
+          <t>• Meta Ads: 71 contas com fonte publicada e execução com sucesso (7 antigas + 64 novas publicadas em 14/10; 7 delas sem veiculação, 0 linhas de insight; 2 de contas desabilitadas na Meta, só histórico). 8 bloqueadas: 7 por 403 ads_read (a conta não está atribuída ao usuário que autorizou) e 1 por erro 400 no stream ads. Outras 6 (Pátio Gourmet e Mari Mari) são ex-clientes e saíram dos bloqueios. 18 rascunhos aguardam OAuth. Conectada não significa dado na Trusted: as novas só entram depois da execução agendada de terça 20/10.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• Google Ads: 41 contas conectadas. As 14 que falharam por cota 429 em 14/10 voltaram a ter sucesso em 16/10, e a Prestex (OzfZ) também (dado até 12/10, ainda fora da Trusted). 12 pendentes: os rascunhos de 05/10 foram removidos da lista da Nekt (só o H3hJ restou), então precisam de confirmação de que a conta ainda é cliente. 3 bloqueadas: Santo Remédio (AMd2, conta saiu do MCC), Comac e Braga Venda Direta (IDs que não aparecem no MCC).</t>
+          <t>• Google Ads: 41 contas conectadas. As 14 que falharam por cota 429 em 14/10 voltaram a ter sucesso em 16/10, e a Prestex (OzfZ) também (dado até 12/10, ainda fora da Trusted). 10 pendentes (as 2 contas Pátio Gourmet saíram: ex-cliente): os rascunhos de 05/10 foram removidos da lista da Nekt (só o H3hJ restou), então precisam de confirmação de que a conta ainda é cliente. 3 bloqueadas: Santo Remédio (AMd2, conta saiu do MCC), Comac e Braga Venda Direta (IDs que não aparecem no MCC). Santo Remédio (513-801-6841): o e-mail do João de 30/09 diz para não conectar a conta de backup por ora; não autorizar sem confirmação.</t>
         </is>
       </c>
     </row>
@@ -891,14 +893,14 @@
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2) Administrador do Business Manager Meta: atribuir ao usuário que autorizou a Nekt as 12 contas com 403 (7 delas ainda fora do Business Manager, do Termo) e autorizar o OAuth dos 18 rascunhos restantes. Prazo: antes de 20/10.</t>
+          <t>2) Administrador do Business Manager Meta: atribuir ao usuário que autorizou a Nekt as 7 contas com 403 (Pátio Gourmet e Mari Mari saíram, ex-clientes; Shizen depende de aprovação do cliente, segundo o e-mail do João de 15/10) e autorizar o OAuth dos 18 rascunhos restantes. Prazo: antes de 20/10.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>3) Suporte da Nekt: restaurar a fonte Meta arquivada em 03/09 que continua no escopo (Pátio Gourmet Lojas, uJNk).</t>
+          <t>3) Suporte da Nekt: não há mais restauração pendente (Pátio Gourmet Lojas, uJNk, saiu: ex-cliente).</t>
         </is>
       </c>
     </row>
@@ -1016,12 +1018,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Atribuir ao usuário que autorizou a Nekt as 12 contas com 403 e autorizar o OAuth dos 18 rascunhos Meta; corrigir o anúncio da CA Braga Motos 2</t>
+          <t>Atribuir ao usuário que autorizou a Nekt as 7 contas com 403 (Pátio Gourmet e Mari Mari saíram: ex-clientes) e autorizar o OAuth dos 18 rascunhos Meta; corrigir o anúncio da CA Braga Motos 2</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>12 com 403 + 18 rascunhos + 1 (bU6W)</t>
+          <t>7 com 403 + 18 rascunhos + 1 (bU6W)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1057,12 +1059,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Confirmar quais das 12 contas pendentes ainda são clientes; autorizar OAuth; reautorizar conector v2.53 (23/10); desvincular as 5 contas Nova Era</t>
+          <t>Confirmar quais das 10 contas pendentes (Pátio Gourmet saiu) ainda são clientes; autorizar OAuth; reautorizar conector v2.53 (23/10); desvincular as 5 contas Nova Era; Santo Remédio: não autorizar sem o João confirmar (e-mail de 30/09)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>12 pendentes + 43 fontes (v2.53) + 5 Nova Era</t>
+          <t>10 pendentes + 43 fontes (v2.53) + 5 Nova Era</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1093,17 +1095,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Suporte da Nekt</t>
+          <t>Suporte da Nekt (CANCELADO)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Restaurar facebook-ads-uJNk (Pátio Gourmet Lojas) arquivada em 03/09, depois da atribuição da conta</t>
+          <t>Não pedir mais a restauração da facebook-ads-uJNk: Pátio Gourmet é ex-cliente (16/10)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1177,7 +1179,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>11 + 10</t>
+          <t>9 + 7</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1317,6 +1319,7 @@
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -2169,12 +2172,12 @@
       </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>Pendente — o rascunho não aparece mais na lista da Nekt (arquivado ou excluído em 14–15/10)</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte/rascunho não deve ser mantido</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
@@ -2184,12 +2187,12 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Conta sem fonte na Nekt hoje</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>Account Manager (confirmar se a conta ainda é cliente)</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr"/>
@@ -2202,15 +2205,15 @@
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
-        </is>
-      </c>
-      <c r="T9" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="U9" s="7" t="inlineStr"/>
+          <t>Não integrar. Arquivar a fonte na interface da Nekt (o MCP não arquiva); o 403 deixou de ser pendência</t>
+        </is>
+      </c>
+      <c r="T9" s="7" t="n"/>
+      <c r="U9" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -2258,12 +2261,12 @@
       </c>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Pendente — o rascunho não aparece mais na lista da Nekt (arquivado ou excluído em 14–15/10)</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte/rascunho não deve ser mantido</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
@@ -2273,12 +2276,12 @@
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>Conta sem fonte na Nekt hoje</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>Account Manager (confirmar se a conta ainda é cliente)</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O10" s="7" t="inlineStr"/>
@@ -2291,15 +2294,15 @@
       <c r="R10" s="7" t="inlineStr"/>
       <c r="S10" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
-        </is>
-      </c>
-      <c r="T10" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="U10" s="7" t="inlineStr"/>
+          <t>Não integrar. Arquivar a fonte na interface da Nekt (o MCP não arquiva); o 403 deixou de ser pendência</t>
+        </is>
+      </c>
+      <c r="T10" s="7" t="n"/>
+      <c r="U10" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -2388,15 +2391,15 @@
       </c>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
-        </is>
-      </c>
-      <c r="T11" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="U11" s="7" t="inlineStr"/>
+          <t>NÃO autorizar nem publicar até o João confirmar que o bloqueio estabilizou (e-mail de 30/09: conta de backup não será conectada à Nekt por enquanto)</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="n"/>
+      <c r="U11" s="7" t="inlineStr">
+        <is>
+          <t>Rascunho z1CZ foi autorizado em 15/10 10:08 e excluído em 15/10 11:32 por outra pessoa. Plataforma do e-mail do João não é informada.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -12596,12 +12599,12 @@
       <c r="I122" s="7" t="inlineStr"/>
       <c r="J122" s="10" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K122" s="7" t="inlineStr">
         <is>
-          <t>Bloqueada — publicada, 403 ads_read: a conta não está atribuída ao usuário que autorizou a conexão</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte/rascunho não deve ser mantido</t>
         </is>
       </c>
       <c r="L122" s="7" t="inlineStr">
@@ -12611,12 +12614,12 @@
       </c>
       <c r="M122" s="7" t="inlineStr">
         <is>
-          <t>Atribuir a conta ao usuário que autorizou a Nekt; a fonte desativa após 3 falhas seguidas (27/10)</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N122" s="7" t="inlineStr">
         <is>
-          <t>Admin do BM Meta (a confirmar)</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O122" s="7" t="inlineStr"/>
@@ -12625,15 +12628,15 @@
       <c r="R122" s="7" t="inlineStr"/>
       <c r="S122" s="7" t="inlineStr">
         <is>
-          <t>Atribuir a conta no Business Manager e pedir nova execução</t>
-        </is>
-      </c>
-      <c r="T122" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="U122" s="7" t="inlineStr"/>
+          <t>Não integrar. Arquivar a fonte na interface da Nekt (o MCP não arquiva); o 403 deixou de ser pendência</t>
+        </is>
+      </c>
+      <c r="T122" s="7" t="n"/>
+      <c r="U122" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -12675,12 +12678,12 @@
       <c r="I123" s="7" t="inlineStr"/>
       <c r="J123" s="10" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K123" s="7" t="inlineStr">
         <is>
-          <t>Bloqueada — publicada, 403 ads_read: a conta não está atribuída ao usuário que autorizou a conexão</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte/rascunho não deve ser mantido</t>
         </is>
       </c>
       <c r="L123" s="7" t="inlineStr">
@@ -12690,12 +12693,12 @@
       </c>
       <c r="M123" s="7" t="inlineStr">
         <is>
-          <t>Atribuir a conta ao usuário que autorizou a Nekt; a fonte desativa após 3 falhas seguidas (27/10)</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N123" s="7" t="inlineStr">
         <is>
-          <t>Admin do BM Meta (a confirmar)</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O123" s="7" t="inlineStr"/>
@@ -12704,15 +12707,15 @@
       <c r="R123" s="7" t="inlineStr"/>
       <c r="S123" s="7" t="inlineStr">
         <is>
-          <t>Atribuir a conta no Business Manager e pedir nova execução</t>
-        </is>
-      </c>
-      <c r="T123" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="U123" s="7" t="inlineStr"/>
+          <t>Não integrar. Arquivar a fonte na interface da Nekt (o MCP não arquiva); o 403 deixou de ser pendência</t>
+        </is>
+      </c>
+      <c r="T123" s="7" t="n"/>
+      <c r="U123" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -13949,12 +13952,12 @@
       <c r="I137" s="7" t="inlineStr"/>
       <c r="J137" s="10" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K137" s="7" t="inlineStr">
         <is>
-          <t>Bloqueada — publicada, 403 ads_read: a conta não está atribuída ao usuário que autorizou a conexão</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte/rascunho não deve ser mantido</t>
         </is>
       </c>
       <c r="L137" s="7" t="inlineStr">
@@ -13964,12 +13967,12 @@
       </c>
       <c r="M137" s="7" t="inlineStr">
         <is>
-          <t>Atribuir a conta ao usuário que autorizou a Nekt; a fonte desativa após 3 falhas seguidas (27/10)</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N137" s="7" t="inlineStr">
         <is>
-          <t>Admin do BM Meta (a confirmar)</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O137" s="7" t="inlineStr"/>
@@ -13982,15 +13985,15 @@
       <c r="R137" s="7" t="inlineStr"/>
       <c r="S137" s="7" t="inlineStr">
         <is>
-          <t>Atribuir a conta no Business Manager e pedir nova execução</t>
-        </is>
-      </c>
-      <c r="T137" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="U137" s="7" t="inlineStr"/>
+          <t>Não integrar. Arquivar a fonte na interface da Nekt (o MCP não arquiva); o 403 deixou de ser pendência</t>
+        </is>
+      </c>
+      <c r="T137" s="7" t="n"/>
+      <c r="U137" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -14032,12 +14035,12 @@
       <c r="I138" s="7" t="inlineStr"/>
       <c r="J138" s="10" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K138" s="7" t="inlineStr">
         <is>
-          <t>Bloqueada — publicada, 403 ads_read: a conta não está atribuída ao usuário que autorizou a conexão</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte/rascunho não deve ser mantido</t>
         </is>
       </c>
       <c r="L138" s="7" t="inlineStr">
@@ -14047,12 +14050,12 @@
       </c>
       <c r="M138" s="7" t="inlineStr">
         <is>
-          <t>Atribuir a conta ao usuário que autorizou a Nekt; a fonte desativa após 3 falhas seguidas (27/10)</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N138" s="7" t="inlineStr">
         <is>
-          <t>Admin do BM Meta (a confirmar)</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O138" s="7" t="inlineStr"/>
@@ -14065,15 +14068,15 @@
       <c r="R138" s="7" t="inlineStr"/>
       <c r="S138" s="7" t="inlineStr">
         <is>
-          <t>Atribuir a conta no Business Manager e pedir nova execução</t>
-        </is>
-      </c>
-      <c r="T138" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="U138" s="7" t="inlineStr"/>
+          <t>Não integrar. Arquivar a fonte na interface da Nekt (o MCP não arquiva); o 403 deixou de ser pendência</t>
+        </is>
+      </c>
+      <c r="T138" s="7" t="n"/>
+      <c r="U138" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -14115,12 +14118,12 @@
       <c r="I139" s="7" t="inlineStr"/>
       <c r="J139" s="10" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K139" s="7" t="inlineStr">
         <is>
-          <t>Bloqueada — publicada, 403 ads_read: a conta não está atribuída ao usuário que autorizou a conexão</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte/rascunho não deve ser mantido</t>
         </is>
       </c>
       <c r="L139" s="7" t="inlineStr">
@@ -14130,12 +14133,12 @@
       </c>
       <c r="M139" s="7" t="inlineStr">
         <is>
-          <t>Atribuir a conta ao usuário que autorizou a Nekt; a fonte desativa após 3 falhas seguidas (27/10)</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N139" s="7" t="inlineStr">
         <is>
-          <t>Admin do BM Meta (a confirmar)</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O139" s="7" t="inlineStr"/>
@@ -14148,15 +14151,15 @@
       <c r="R139" s="7" t="inlineStr"/>
       <c r="S139" s="7" t="inlineStr">
         <is>
-          <t>Atribuir a conta no Business Manager e pedir nova execução</t>
-        </is>
-      </c>
-      <c r="T139" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="U139" s="7" t="inlineStr"/>
+          <t>Não integrar. Arquivar a fonte na interface da Nekt (o MCP não arquiva); o 403 deixou de ser pendência</t>
+        </is>
+      </c>
+      <c r="T139" s="7" t="n"/>
+      <c r="U139" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -16155,12 +16158,12 @@
       <c r="I161" s="7" t="inlineStr"/>
       <c r="J161" s="11" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K161" s="7" t="inlineStr">
         <is>
-          <t>Bloqueada — fonte arquivada em 03/09 (perdeu permissão ads_read, erro 403 #200)</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte/rascunho não deve ser mantido</t>
         </is>
       </c>
       <c r="L161" s="7" t="inlineStr">
@@ -16170,12 +16173,12 @@
       </c>
       <c r="M161" s="7" t="inlineStr">
         <is>
-          <t>Restaurar fonte arquivada exige o suporte da Nekt; token precisa de ads_read na conta</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N161" s="7" t="inlineStr">
         <is>
-          <t>Suporte Nekt + admin do BM Meta</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O161" s="7" t="inlineStr"/>
@@ -16188,15 +16191,15 @@
       <c r="R161" s="7" t="inlineStr"/>
       <c r="S161" s="7" t="inlineStr">
         <is>
-          <t>Pedir restauração ao suporte e re-autorizar com usuário que tenha a conta</t>
-        </is>
-      </c>
-      <c r="T161" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="U161" s="7" t="inlineStr"/>
+          <t>Não integrar. Arquivar a fonte na interface da Nekt (o MCP não arquiva); o 403 deixou de ser pendência</t>
+        </is>
+      </c>
+      <c r="T161" s="7" t="n"/>
+      <c r="U161" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -22616,12 +22619,12 @@
       <c r="I236" s="7" t="inlineStr"/>
       <c r="J236" s="14" t="inlineStr">
         <is>
-          <t>Sem conexão</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K236" s="7" t="inlineStr">
         <is>
-          <t>Sem conexão — não há conector Nekt para esta plataforma</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte/rascunho não deve ser mantido</t>
         </is>
       </c>
       <c r="L236" s="7" t="inlineStr">
@@ -22631,12 +22634,12 @@
       </c>
       <c r="M236" s="7" t="inlineStr">
         <is>
-          <t>ID da conta não consta em nenhum documento</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N236" s="7" t="inlineStr">
         <is>
-          <t>Analista da conta</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O236" s="7" t="inlineStr"/>
@@ -22649,15 +22652,15 @@
       <c r="R236" s="7" t="inlineStr"/>
       <c r="S236" s="7" t="inlineStr">
         <is>
-          <t>Levantar ID da conta e decidir se entra no escopo</t>
-        </is>
-      </c>
-      <c r="T236" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="U236" s="7" t="inlineStr"/>
+          <t>Não integrar. Arquivar a fonte na interface da Nekt (o MCP não arquiva); o 403 deixou de ser pendência</t>
+        </is>
+      </c>
+      <c r="T236" s="7" t="n"/>
+      <c r="U236" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="7" t="inlineStr">
@@ -22794,12 +22797,12 @@
       <c r="I238" s="7" t="inlineStr"/>
       <c r="J238" s="14" t="inlineStr">
         <is>
-          <t>Sem conexão</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K238" s="7" t="inlineStr">
         <is>
-          <t>Sem conexão — conector tiktok-ads existe na Nekt, nenhuma fonte criada</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte/rascunho não deve ser mantido</t>
         </is>
       </c>
       <c r="L238" s="7" t="inlineStr">
@@ -22809,12 +22812,12 @@
       </c>
       <c r="M238" s="7" t="inlineStr">
         <is>
-          <t>ID da conta não consta em nenhum documento</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N238" s="7" t="inlineStr">
         <is>
-          <t>Analista da conta</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O238" s="7" t="inlineStr"/>
@@ -22827,15 +22830,15 @@
       <c r="R238" s="7" t="inlineStr"/>
       <c r="S238" s="7" t="inlineStr">
         <is>
-          <t>Levantar ID da conta e decidir se entra no escopo</t>
-        </is>
-      </c>
-      <c r="T238" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="U238" s="7" t="inlineStr"/>
+          <t>Não integrar. Arquivar a fonte na interface da Nekt (o MCP não arquiva); o 403 deixou de ser pendência</t>
+        </is>
+      </c>
+      <c r="T238" s="7" t="n"/>
+      <c r="U238" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="7" t="inlineStr">
@@ -23055,12 +23058,12 @@
       <c r="I241" s="7" t="inlineStr"/>
       <c r="J241" s="14" t="inlineStr">
         <is>
-          <t>Sem conexão</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K241" s="7" t="inlineStr">
         <is>
-          <t>Sem conexão — não há conector Nekt para esta plataforma</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte/rascunho não deve ser mantido</t>
         </is>
       </c>
       <c r="L241" s="7" t="inlineStr">
@@ -23070,12 +23073,12 @@
       </c>
       <c r="M241" s="7" t="inlineStr">
         <is>
-          <t>ID da conta não consta em nenhum documento</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N241" s="7" t="inlineStr">
         <is>
-          <t>Analista da conta</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O241" s="7" t="inlineStr"/>
@@ -23088,15 +23091,15 @@
       <c r="R241" s="7" t="inlineStr"/>
       <c r="S241" s="7" t="inlineStr">
         <is>
-          <t>Levantar ID da conta e decidir se entra no escopo</t>
-        </is>
-      </c>
-      <c r="T241" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="U241" s="7" t="inlineStr"/>
+          <t>Não integrar. Arquivar a fonte na interface da Nekt (o MCP não arquiva); o 403 deixou de ser pendência</t>
+        </is>
+      </c>
+      <c r="T241" s="7" t="n"/>
+      <c r="U241" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:U241"/>
@@ -23110,7 +23113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23216,11 +23219,11 @@
         </is>
       </c>
       <c r="E3" s="7" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>ARENA TINTAS [E-COM + AQUISIÇÃO]; BA ELÉTRICA; FARMABEM; MARI MARI; PÁTIO GOURMET [E-COM]; PÁTIO GOURMET [LOJAS]; SANTO REMÉDIO; SHIZEN</t>
+          <t>ARENA TINTAS [E-COM + AQUISIÇÃO]; BA ELÉTRICA; FARMABEM; SANTO REMÉDIO; SHIZEN</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -23286,11 +23289,11 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>AÇO MANAUS; BRAGA MOTORS BMW; CDL MANAUS; DR. CABRAL (conta 2 NOVA); HOPE BAY PARK; JULIA HERRERA; PÁTIO GOURMET (E-COM); PÁTIO GOURMET (LOJA); SANTO REMÉDIO (conta viva); TUBOAÇOS DA AMAZÔNIA; UIARA AMAZON RESORT</t>
+          <t>AÇO MANAUS; BRAGA MOTORS BMW; CDL MANAUS; DR. CABRAL (conta 2 NOVA); HOPE BAY PARK; JULIA HERRERA; SANTO REMÉDIO (conta viva); TUBOAÇOS DA AMAZÔNIA; UIARA AMAZON RESORT</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -23622,17 +23625,17 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>RD Station</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Suporte Nekt + admin do BM Meta</t>
+          <t>Analista Inbound (Bryan) + admin da conta RD do CDL</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Pedir restauração ao suporte e re-autorizar com usuário que tenha a conta</t>
+          <t>Conferir plano/permissão da conta RD do CDL e reautorizar</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
@@ -23640,7 +23643,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>PÁTIO GOURMET [LOJAS]</t>
+          <t>CDL</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -23662,25 +23665,25 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound (Bryan) + admin da conta RD do CDL</t>
+          <t>Analista Inbound (Bryan) + admin da conta RD do cliente (a confirmar)</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Conferir plano/permissão da conta RD do CDL e reautorizar</t>
+          <t>Analista Inbound confirmar se a conta RD existe; se sim, recriar o rascunho</t>
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>CDL</t>
+          <t>LEGACY PNEUS; LOVOL; TARGO CONSULTORIA</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Pendente</t>
         </is>
       </c>
     </row>
@@ -23697,20 +23700,20 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound (Bryan) + admin da conta RD do cliente (a confirmar)</t>
+          <t>Analista Inbound (Joyce) + admin da conta RD do cliente (a confirmar)</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound confirmar se a conta RD existe; se sim, recriar o rascunho</t>
+          <t>Encaminhar link de autorização ao administrador da conta RD</t>
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>LEGACY PNEUS; LOVOL; TARGO CONSULTORIA</t>
+          <t>BRAGA MOTOS - YAMAHA - VENDAS</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -23732,12 +23735,12 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound (Joyce) + admin da conta RD do cliente (a confirmar)</t>
+          <t>Analista Inbound (Juan Carlos) + admin da conta RD do cliente (a confirmar)</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Encaminhar link de autorização ao administrador da conta RD</t>
+          <t>Analista Inbound confirmar se a conta RD existe; se sim, recriar o rascunho</t>
         </is>
       </c>
       <c r="E18" s="7" t="n">
@@ -23745,7 +23748,7 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>BRAGA MOTOS - YAMAHA - VENDAS</t>
+          <t>BRAGA VEÍCULOS VENDAS - PÓS VENDA</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -23767,12 +23770,12 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound (Juan Carlos) + admin da conta RD do cliente (a confirmar)</t>
+          <t>Jussara (diagnóstico na Nekt) + Analista Inbound (Joyce)</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound confirmar se a conta RD existe; se sim, recriar o rascunho</t>
+          <t>Conferir se a conta RD do cliente tem contatos/conversões e a permissão da API</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -23780,12 +23783,12 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>BRAGA VEÍCULOS VENDAS - PÓS VENDA</t>
+          <t>AMZ IMPORTS</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Conectada</t>
         </is>
       </c>
     </row>
@@ -23802,20 +23805,20 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Jussara (diagnóstico na Nekt) + Analista Inbound (Joyce)</t>
+          <t>Nekt (Jussara)</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Conferir se a conta RD do cliente tem contatos/conversões e a permissão da API</t>
+          <t>Conferir carga e somar às Trusted de RD</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>AMZ IMPORTS</t>
+          <t>ARENA TINTAS; BAJAJ; BAP; BRAGA MOTOS - YAMAHA - PÓS VENDAS; BRAGA VEÍCULOS - VENDA DIRETA; BRAGA VEÍCULOS VAREJO; CAA ALUMÍNIO; CAA TINTAS; CHARÃO; CONSTROI INCORPORADORA; DISTRIBUIDORA PNEU FORTE; DOCTOR MAIS SAÚDE; HAGE ALIMENTOS; PMZ ESCOLA; RODRIX; ROYAL ENFIELD; SANTO REMÉDIO; SHIZEN; UNIPAR</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -23827,30 +23830,30 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>RD Station</t>
+          <t>Google Ads</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Nekt (Jussara)</t>
+          <t>Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Conferir carga e somar às Trusted de RD</t>
+          <t>Reautorizar no prazo da Google (23/10)</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>ARENA TINTAS; BAJAJ; BAP; BRAGA MOTOS - YAMAHA - PÓS VENDAS; BRAGA VEÍCULOS - VENDA DIRETA; BRAGA VEÍCULOS VAREJO; CAA ALUMÍNIO; CAA TINTAS; CHARÃO; CONSTROI INCORPORADORA; DISTRIBUIDORA PNEU FORTE; DOCTOR MAIS SAÚDE; HAGE ALIMENTOS; PMZ ESCOLA; RODRIX; ROYAL ENFIELD; SANTO REMÉDIO; SHIZEN; UNIPAR</t>
+          <t>ACESSO SAÚDE; AMAZONCOPY; AMZ GERADORES; ARENA TINTAS; BA ELÉTRICA; BIGAZINE; CAA ALUMÍNIO; CAA TINTAS; COLMEIA; CONSTRÓI INCORPORADORA; DEB TRANSPORTADORA; DOCTOR MAIS; DON WATCHES (conta 2); HOSPITAL SANTA JÚLIA; MILLENIUM; MOVE RENTAL CARS; OLÁ CASA NOVA; PMZ ESCOLA DE MECÂNICOS; PMZ GRUPO ECOMM; PMZ GRUPO LOJA; PNEU EXPRESS; PNEU FORTE DISTRIBUIDORA; REI DAS MANGUEIRAS; RODRIX; SMILE PNEUS; STEEL PORT</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -23872,60 +23875,60 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
+          <t>Jussara + administrador do MCC</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Reautorizar no prazo da Google (23/10)</t>
+          <t>Não integrar; solicitar desvínculo da conta do MCC</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>ACESSO SAÚDE; AMAZONCOPY; AMZ GERADORES; ARENA TINTAS; BA ELÉTRICA; BIGAZINE; CAA ALUMÍNIO; CAA TINTAS; COLMEIA; CONSTRÓI INCORPORADORA; DEB TRANSPORTADORA; DOCTOR MAIS; DON WATCHES (conta 2); HOSPITAL SANTA JÚLIA; MILLENIUM; MOVE RENTAL CARS; OLÁ CASA NOVA; PMZ ESCOLA DE MECÂNICOS; PMZ GRUPO ECOMM; PMZ GRUPO LOJA; PNEU EXPRESS; PNEU FORTE DISTRIBUIDORA; REI DAS MANGUEIRAS; RODRIX; SMILE PNEUS; STEEL PORT</t>
+          <t>LOJA | NOVA ERA BV | PIX; LOJA | NOVA ERA PVH | PIX; NOVA ERA MAO | LOJAS; NOVA ERA | MANAUS | ECOMM; NOVA ERA | PORTO VELHO | ECOMM</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Conectada</t>
+          <t>Fora do escopo (Nova Era)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Google Ads</t>
+          <t>LinkedIn Ads</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Jussara + administrador do MCC</t>
+          <t>Analista da conta</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Não integrar; solicitar desvínculo da conta do MCC</t>
+          <t>Levantar ID da conta e decidir se entra no escopo</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>LOJA | NOVA ERA BV | PIX; LOJA | NOVA ERA PVH | PIX; NOVA ERA MAO | LOJAS; NOVA ERA | MANAUS | ECOMM; NOVA ERA | PORTO VELHO | ECOMM</t>
+          <t>ALMEIDA E BARRETO; AMAZONCOPY; PRESTEX; TUBOAÇOS</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Fora do escopo (Nova Era)</t>
+          <t>Sem conexão</t>
         </is>
       </c>
     </row>
@@ -23937,7 +23940,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>LinkedIn Ads</t>
+          <t>TikTok Ads</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -23951,119 +23954,14 @@
         </is>
       </c>
       <c r="E24" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>ALMEIDA E BARRETO; AMAZONCOPY; PRESTEX; TUBOAÇOS</t>
+          <t>BA ELÉTRICA; SANTO REMÉDIO; TUBOAÇOS</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>Sem conexão</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Spotify Ads</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Analista da conta</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Levantar ID da conta e decidir se entra no escopo</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>PÁTIO GOURMET (LOJAS)</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>Sem conexão</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>TikTok Ads</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Analista da conta</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>Levantar ID da conta e decidir se entra no escopo</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>BA ELÉTRICA; PÁTIO GOURMET (LOJAS); SANTO REMÉDIO; TUBOAÇOS</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>Sem conexão</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Twitter/X Ads</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Analista da conta</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Levantar ID da conta e decidir se entra no escopo</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>PÁTIO GOURMET (LOJAS)</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>Sem conexão</t>
         </is>
@@ -24081,7 +23979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -24197,11 +24095,11 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Atribuir a conta no Business Manager e pedir nova execução (12)</t>
+          <t>Atribuir a conta no Business Manager e pedir nova execução (7)</t>
         </is>
       </c>
       <c r="D4" s="7" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -24227,11 +24125,11 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth (11)</t>
+          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth (9)</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
@@ -24257,11 +24155,11 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Levantar ID da conta e decidir se entra no escopo (10)</t>
+          <t>Levantar ID da conta e decidir se entra no escopo (7)</t>
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
@@ -24505,7 +24403,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Suporte Nekt + admin do BM Meta</t>
+          <t>Analista Inbound (Joyce) + admin da conta RD do cliente (a confirmar)</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -24515,7 +24413,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Pedir restauração ao suporte e re-autorizar com usuário que tenha a conta (1)</t>
+          <t>Encaminhar link de autorização ao administrador da conta RD (1)</t>
         </is>
       </c>
       <c r="D15" s="7" t="n">
@@ -24535,7 +24433,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound (Joyce) + admin da conta RD do cliente (a confirmar)</t>
+          <t>Analista Inbound (Juan Carlos) + admin da conta RD do cliente (a confirmar)</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -24545,7 +24443,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Encaminhar link de autorização ao administrador da conta RD (1)</t>
+          <t>Analista Inbound confirmar se a conta RD existe; se sim, recriar o rascunho (1)</t>
         </is>
       </c>
       <c r="D16" s="7" t="n">
@@ -24565,7 +24463,7 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound (Juan Carlos) + admin da conta RD do cliente (a confirmar)</t>
+          <t>Analista Inbound (Bryan) + admin da conta RD do CDL</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -24575,7 +24473,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound confirmar se a conta RD existe; se sim, recriar o rascunho (1)</t>
+          <t>Conferir plano/permissão da conta RD do CDL e reautorizar (1)</t>
         </is>
       </c>
       <c r="D17" s="7" t="n">
@@ -24595,7 +24493,7 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound (Bryan) + admin da conta RD do CDL</t>
+          <t>Jussara (diagnóstico na Nekt) + Analista Inbound (Joyce)</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -24605,7 +24503,7 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Conferir plano/permissão da conta RD do CDL e reautorizar (1)</t>
+          <t>Conferir se a conta RD do cliente tem contatos/conversões e a permissão da API (1)</t>
         </is>
       </c>
       <c r="D18" s="7" t="n">
@@ -24617,36 +24515,6 @@
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>docs/nekt/solicitacoes-1743-2026-10-15.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Jussara (diagnóstico na Nekt) + Analista Inbound (Joyce)</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>E-mail + tarefa no VJOB</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>Conferir se a conta RD do cliente tem contatos/conversões e a permissão da API (1)</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>docs/nekt/solicitacoes-1743-2026-10-15.md</t>
         </is>
@@ -24663,7 +24531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -24802,6 +24670,20 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>• ATUALIZAÇÃO DE 16/10 (tarde): Pátio Gourmet e Mari Mari não são mais clientes da agência (informado pela Jussara). 11 linhas passaram a 'Não precisa manter (ex-cliente)': Meta 6 (Mari Mari x2, Pátio Gourmet x4, incluindo a uJNk arquivada), Google 2 e Spotify, TikTok e X de Pátio Gourmet 1 cada. Os 403 dessas 5 fontes publicadas (gp7f, flYR, bhnp, XuHY, 7vwE) deixam de ser pendência. As fontes continuam publicadas e vão falhar até 27/10, quando a Nekt as desativa; arquivar só é possível na interface da Nekt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>• Santo Remédio: e-mail do João de 30/09 diz que a conta antiga foi bloqueada e que a conta de backup não será conectada à Nekt por ora. A linha Google (513-801-6841) segue 'Pendente' mas com ação 'não autorizar até confirmar'. As fontes Meta f6h8 e geQA (403) não são cobertas pelo e-mail. Shizen: e-mail de 15/10 diz que falta aprovação específica do cliente.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
One pager da #1744 v3: Olá Casa Nova (Meta e Google) sai do escopo
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNtRG1wGaTmzdzTc1r8f3Q
</commit_message>
<xml_diff>
--- a/docs/nekt/inventario-contas-1743-2026-10-16.xlsx
+++ b/docs/nekt/inventario-contas-1743-2026-10-16.xlsx
@@ -545,7 +545,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -595,7 +594,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C5" t="n">
         <v>18</v>
@@ -610,7 +609,7 @@
         <v>8</v>
       </c>
       <c r="G5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5" t="n">
         <v>111</v>
@@ -623,7 +622,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C6" t="n">
         <v>10</v>
@@ -638,7 +637,7 @@
         <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
         <v>61</v>
@@ -819,7 +818,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
@@ -830,14 +828,14 @@
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>• Meta Ads: 71 contas com fonte publicada e execução com sucesso (7 antigas + 64 novas publicadas em 14/10; 7 delas sem veiculação, 0 linhas de insight; 2 de contas desabilitadas na Meta, só histórico). 8 bloqueadas: 7 por 403 ads_read (a conta não está atribuída ao usuário que autorizou) e 1 por erro 400 no stream ads. Outras 6 (Pátio Gourmet e Mari Mari) são ex-clientes e saíram dos bloqueios. 18 rascunhos aguardam OAuth. Conectada não significa dado na Trusted: as novas só entram depois da execução agendada de terça 20/10.</t>
+          <t>• Meta Ads: 70 contas com fonte publicada e execução com sucesso (7 antigas + 63 novas publicadas em 14/10; 6 delas sem veiculação, 0 linhas de insight; 2 de contas desabilitadas na Meta, só histórico). 8 bloqueadas: 7 por 403 ads_read (a conta não está atribuída ao usuário que autorizou) e 1 por erro 400 no stream ads. Outras 6 (Pátio Gourmet e Mari Mari) são ex-clientes e saíram dos bloqueios. 18 rascunhos aguardam OAuth. Conectada não significa dado na Trusted: as novas só entram depois da execução agendada de terça 20/10.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• Google Ads: 41 contas conectadas. As 14 que falharam por cota 429 em 14/10 voltaram a ter sucesso em 16/10, e a Prestex (OzfZ) também (dado até 12/10, ainda fora da Trusted). 10 pendentes (as 2 contas Pátio Gourmet saíram: ex-cliente): os rascunhos de 05/10 foram removidos da lista da Nekt (só o H3hJ restou), então precisam de confirmação de que a conta ainda é cliente. 3 bloqueadas: Santo Remédio (AMd2, conta saiu do MCC), Comac e Braga Venda Direta (IDs que não aparecem no MCC). Santo Remédio (513-801-6841): o e-mail do João de 30/09 diz para não conectar a conta de backup por ora; não autorizar sem confirmação.</t>
+          <t>• Google Ads: 40 contas conectadas (a Olá Casa Nova saiu: ex-cliente). As 14 que falharam por cota 429 em 14/10 voltaram a ter sucesso em 16/10, e a Prestex (OzfZ) também (dado até 12/10, ainda fora da Trusted). 10 pendentes (as 2 contas Pátio Gourmet saíram: ex-cliente): os rascunhos de 05/10 foram removidos da lista da Nekt (só o H3hJ restou), então precisam de confirmação de que a conta ainda é cliente. 3 bloqueadas: Santo Remédio (AMd2, conta saiu do MCC), Comac e Braga Venda Direta (IDs que não aparecem no MCC). Santo Remédio (513-801-6841): o e-mail do João de 30/09 diz para não conectar a conta de backup por ora; não autorizar sem confirmação.</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1317,6 @@
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -5387,12 +5384,12 @@
       <c r="I44" s="7" t="inlineStr"/>
       <c r="J44" s="12" t="inlineStr">
         <is>
-          <t>Conectada</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K44" s="7" t="inlineStr">
         <is>
-          <t>Conectada e extraindo</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte não deve ser mantida</t>
         </is>
       </c>
       <c r="L44" s="7" t="inlineStr">
@@ -5402,12 +5399,12 @@
       </c>
       <c r="M44" s="7" t="inlineStr">
         <is>
-          <t>Reautorização v2.53 do conector até 23/10/2026</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N44" s="7" t="inlineStr">
         <is>
-          <t>Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O44" s="7" t="inlineStr"/>
@@ -5416,15 +5413,15 @@
       <c r="R44" s="7" t="inlineStr"/>
       <c r="S44" s="7" t="inlineStr">
         <is>
-          <t>Reautorizar no prazo da Google (23/10)</t>
-        </is>
-      </c>
-      <c r="T44" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="U44" s="7" t="inlineStr"/>
+          <t>Não integrar mais. Arquivar a fonte na interface da Nekt (o MCP não arquiva)</t>
+        </is>
+      </c>
+      <c r="T44" s="7" t="n"/>
+      <c r="U44" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado. Google: dado até 12/10, R$ 2.208,42 em 13/09–12/10 (conta no MCC: pedir desvínculo ou pausa).</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -13218,12 +13215,12 @@
       <c r="I129" s="7" t="inlineStr"/>
       <c r="J129" s="10" t="inlineStr">
         <is>
-          <t>Conectada</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K129" s="7" t="inlineStr">
         <is>
-          <t>Conectada — publicada, execução com sucesso, sem veiculação na janela (0 linhas de insight)</t>
+          <t>Ex-cliente — a agência não atende mais (informado pela Jussara em 16/10); fonte não deve ser mantida</t>
         </is>
       </c>
       <c r="L129" s="7" t="inlineStr">
@@ -13233,12 +13230,12 @@
       </c>
       <c r="M129" s="7" t="inlineStr">
         <is>
-          <t>Conta sem veiculação; entra dado na 1ª veiculação (limite de gasto pode estar esgotado)</t>
+          <t>Sem pendência de conexão: cliente encerrado</t>
         </is>
       </c>
       <c r="N129" s="7" t="inlineStr">
         <is>
-          <t>AM do cliente</t>
+          <t>Jussara (arquivar na interface da Nekt)</t>
         </is>
       </c>
       <c r="O129" s="7" t="inlineStr"/>
@@ -13247,15 +13244,15 @@
       <c r="R129" s="7" t="inlineStr"/>
       <c r="S129" s="7" t="inlineStr">
         <is>
-          <t>Acompanhar; se o cliente for veicular, renovar o limite na Meta</t>
-        </is>
-      </c>
-      <c r="T129" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="U129" s="7" t="inlineStr"/>
+          <t>Não integrar mais. Arquivar a fonte na interface da Nekt (o MCP não arquiva)</t>
+        </is>
+      </c>
+      <c r="T129" s="7" t="n"/>
+      <c r="U129" s="7" t="inlineStr">
+        <is>
+          <t>Cliente encerrado, confirmado pela Jussara em 16/10/2026. Histórico na Raw preservado.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -23849,11 +23846,11 @@
         </is>
       </c>
       <c r="E21" s="7" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>ACESSO SAÚDE; AMAZONCOPY; AMZ GERADORES; ARENA TINTAS; BA ELÉTRICA; BIGAZINE; CAA ALUMÍNIO; CAA TINTAS; COLMEIA; CONSTRÓI INCORPORADORA; DEB TRANSPORTADORA; DOCTOR MAIS; DON WATCHES (conta 2); HOSPITAL SANTA JÚLIA; MILLENIUM; MOVE RENTAL CARS; OLÁ CASA NOVA; PMZ ESCOLA DE MECÂNICOS; PMZ GRUPO ECOMM; PMZ GRUPO LOJA; PNEU EXPRESS; PNEU FORTE DISTRIBUIDORA; REI DAS MANGUEIRAS; RODRIX; SMILE PNEUS; STEEL PORT</t>
+          <t>ACESSO SAÚDE; AMAZONCOPY; AMZ GERADORES; ARENA TINTAS; BA ELÉTRICA; BIGAZINE; CAA ALUMÍNIO; CAA TINTAS; COLMEIA; CONSTRÓI INCORPORADORA; DEB TRANSPORTADORA; DOCTOR MAIS; DON WATCHES (conta 2); HOSPITAL SANTA JÚLIA; MILLENIUM; MOVE RENTAL CARS; PMZ ESCOLA DE MECÂNICOS; PMZ GRUPO ECOMM; PMZ GRUPO LOJA; PNEU EXPRESS; PNEU FORTE DISTRIBUIDORA; REI DAS MANGUEIRAS; RODRIX; SMILE PNEUS; STEEL PORT</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -24035,11 +24032,11 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Reautorizar no prazo da Google (23/10) (26); Encaminhar link de autorização ao administrador do MCC (1); Reautorizar a fonte OzfZ (1); Encerrar a AMd2 na interface depois de integrar a conta viva; histórico preservado (1); Integrar a conta NOVA e então decidir encerrar a wypN (1)</t>
+          <t>Reautorizar no prazo da Google (23/10) (25); Encaminhar link de autorização ao administrador do MCC (1); Reautorizar a fonte OzfZ (1); Encerrar a AMd2 na interface depois de integrar a conta viva; histórico preservado (1); Integrar a conta NOVA e então decidir encerrar a wypN (1)</t>
         </is>
       </c>
       <c r="D2" s="7" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
@@ -24531,7 +24528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -24684,6 +24681,13 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>• ATUALIZAÇÃO DE 16/10 (fim da tarde): Olá Casa Nova também saiu (ex-cliente, informado pela Jussara). 2 linhas: Meta (facebook-ads-FKfU, conectada com 0 linhas, a que era a única 'conectada sem confirmação') e Google (google-ads-DzVL, conectada com dado até 12/10). Efeito no one pager da #1744: aplicáveis 153 → 151, confirmadas 112 → 111. A reautorização v2.53 (23/10) não precisa mais cobrir a google-ads-DzVL. Arquivar as duas fontes é pela interface da Nekt.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Planilha oficial #1743: acrescenta Dmello e conta própria da Vanguarda (Google)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNtRG1wGaTmzdzTc1r8f3Q
</commit_message>
<xml_diff>
--- a/docs/nekt/inventario-contas-1743-2026-10-16.xlsx
+++ b/docs/nekt/inventario-contas-1743-2026-10-16.xlsx
@@ -622,10 +622,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6" t="n">
         <v>3</v>
@@ -640,7 +640,7 @@
         <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7">
@@ -1335,7 +1335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U241"/>
+  <dimension ref="A1:U243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23098,6 +23098,182 @@
         </is>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" s="7" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="B242" s="7" t="inlineStr">
+        <is>
+          <t>DMELLO (TEMPO DAS TINTAS)</t>
+        </is>
+      </c>
+      <c r="C242" s="8" t="inlineStr">
+        <is>
+          <t>331-057-9239</t>
+        </is>
+      </c>
+      <c r="D242" s="7" t="inlineStr">
+        <is>
+          <t>Dmello Tempo das Tintas</t>
+        </is>
+      </c>
+      <c r="E242" s="7" t="inlineStr">
+        <is>
+          <t>Acrescentada em 16/10 (já estava no inventário de fontes de 15/10)</t>
+        </is>
+      </c>
+      <c r="F242" s="7" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="G242" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H242" s="9" t="n"/>
+      <c r="I242" s="7" t="inlineStr">
+        <is>
+          <t>BRL</t>
+        </is>
+      </c>
+      <c r="J242" s="11" t="inlineStr">
+        <is>
+          <t>Conectada</t>
+        </is>
+      </c>
+      <c r="K242" s="7" t="inlineStr">
+        <is>
+          <t>Conectada e extraindo (leitura confirmada; conta parada)</t>
+        </is>
+      </c>
+      <c r="L242" s="7" t="inlineStr">
+        <is>
+          <t>google-ads-URNQ</t>
+        </is>
+      </c>
+      <c r="M242" s="7" t="inlineStr">
+        <is>
+          <t>Reautorização v2.53 do conector até 23/10/2026</t>
+        </is>
+      </c>
+      <c r="N242" s="7" t="inlineStr">
+        <is>
+          <t>Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
+        </is>
+      </c>
+      <c r="O242" s="7" t="n"/>
+      <c r="P242" s="7" t="n"/>
+      <c r="Q242" s="7" t="n"/>
+      <c r="R242" s="7" t="n"/>
+      <c r="S242" s="7" t="inlineStr">
+        <is>
+          <t>Reautorizar no prazo da Google (23/10)</t>
+        </is>
+      </c>
+      <c r="T242" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="U242" s="7" t="inlineStr">
+        <is>
+          <t>Faltava no inventário #1743 oficial; corrigido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="7" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="B243" s="7" t="inlineStr">
+        <is>
+          <t>VANGUARDA COMUNICAÇÃO (conta própria)</t>
+        </is>
+      </c>
+      <c r="C243" s="8" t="inlineStr">
+        <is>
+          <t>750-265-3880</t>
+        </is>
+      </c>
+      <c r="D243" s="7" t="inlineStr">
+        <is>
+          <t>Vanguarda</t>
+        </is>
+      </c>
+      <c r="E243" s="7" t="inlineStr">
+        <is>
+          <t>Acrescentada em 16/10 (já estava no inventário de fontes de 15/10)</t>
+        </is>
+      </c>
+      <c r="F243" s="7" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="G243" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H243" s="9" t="n">
+        <v>161.26</v>
+      </c>
+      <c r="I243" s="7" t="inlineStr">
+        <is>
+          <t>BRL</t>
+        </is>
+      </c>
+      <c r="J243" s="10" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K243" s="7" t="inlineStr">
+        <is>
+          <t>Pendente — conta própria da agência com gasto e sem fonte</t>
+        </is>
+      </c>
+      <c r="L243" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M243" s="7" t="inlineStr">
+        <is>
+          <t>Conta sem fonte na Nekt hoje (a Meta da Vanguarda já está conectada)</t>
+        </is>
+      </c>
+      <c r="N243" s="7" t="inlineStr">
+        <is>
+          <t>Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
+        </is>
+      </c>
+      <c r="O243" s="7" t="n"/>
+      <c r="P243" s="7" t="n"/>
+      <c r="Q243" s="7" t="n"/>
+      <c r="R243" s="7" t="n"/>
+      <c r="S243" s="7" t="inlineStr">
+        <is>
+          <t>Decidir se entra; se sim, criar o rascunho e pedir o OAuth</t>
+        </is>
+      </c>
+      <c r="T243" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="U243" s="7" t="inlineStr">
+        <is>
+          <t>Faltava no inventário #1743 oficial; corrigido. Gasto 13/09–12/10.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:U241"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24528,7 +24704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -24688,6 +24864,13 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>• CORREÇÃO DE 16/10: duas contas Google que já constavam no inventário de fontes de 15/10 faltavam nesta planilha e foram acrescentadas: Dmello (google-ads-URNQ, 331-057-9239, conectada) e a conta própria da Vanguarda (750-265-3880, pendente, R$ 161,26 em 13/09–12/10). O Resumo do Google passa a 41 conectadas e 11 pendentes.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
One pager da #1744 v4 e planilha oficial: status das 10 contas Google pendentes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNtRG1wGaTmzdzTc1r8f3Q
</commit_message>
<xml_diff>
--- a/docs/nekt/inventario-contas-1743-2026-10-16.xlsx
+++ b/docs/nekt/inventario-contas-1743-2026-10-16.xlsx
@@ -578,7 +578,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Não precisa manter (ex-cliente / duplicata)</t>
+          <t>Não precisa manter (ex-cliente, duplicidade ou decisão)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -625,10 +625,10 @@
         <v>41</v>
       </c>
       <c r="C6" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -637,7 +637,7 @@
         <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H6" t="n">
         <v>63</v>
@@ -818,6 +818,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
@@ -1057,12 +1058,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Confirmar quais das 10 contas pendentes (Pátio Gourmet saiu) ainda são clientes; autorizar OAuth; reautorizar conector v2.53 (23/10); desvincular as 5 contas Nova Era; Santo Remédio: não autorizar sem o João confirmar (e-mail de 30/09)</t>
+          <t>Reautorizar conector v2.53 (23/10); autorizar OAuth das 4 contas que aguardam autorização (Aço Manaus, Braga Motors BMW, Pneu Forte Varejo, Tuboaços); desvincular ou pausar as contas de ex-clientes (5 Nova Era, 2 Pátio Gourmet, Olá Casa Nova, Hope Bay Park, Julia Herrera, UIARA)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>10 pendentes + 43 fontes (v2.53) + 5 Nova Era</t>
+          <t>4 aguardando autorização + 42 fontes (v2.53) + 11 desvínculos</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1317,6 +1318,7 @@
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -1519,7 +1521,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>Pendente — o rascunho não aparece mais na lista da Nekt (arquivado ou excluído em 14–15/10)</t>
+          <t>Pendente — aguardando autorização (informado pela jussara em 16/10)</t>
         </is>
       </c>
       <c r="L2" s="7" t="inlineStr">
@@ -1529,7 +1531,7 @@
       </c>
       <c r="M2" s="7" t="inlineStr">
         <is>
-          <t>Conta sem fonte na Nekt hoje</t>
+          <t>Aguardando autorização (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="N2" s="7" t="inlineStr">
@@ -1547,14 +1549,10 @@
       <c r="R2" s="7" t="inlineStr"/>
       <c r="S2" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
-        </is>
-      </c>
-      <c r="T2" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>Aguardar a autorização do cliente/administrador; depois OAuth e publicar</t>
+        </is>
+      </c>
+      <c r="T2" s="7" t="n"/>
       <c r="U2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
@@ -1608,7 +1606,7 @@
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Pendente — o rascunho não aparece mais na lista da Nekt (arquivado ou excluído em 14–15/10)</t>
+          <t>Pendente — aguardando autorização (informado pela jussara em 16/10)</t>
         </is>
       </c>
       <c r="L3" s="7" t="inlineStr">
@@ -1618,7 +1616,7 @@
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>Conta sem fonte na Nekt hoje</t>
+          <t>Aguardando autorização (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
@@ -1648,14 +1646,10 @@
       </c>
       <c r="S3" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
-        </is>
-      </c>
-      <c r="T3" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>Aguardar a autorização do cliente/administrador; depois OAuth e publicar</t>
+        </is>
+      </c>
+      <c r="T3" s="7" t="n"/>
       <c r="U3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
@@ -1704,12 +1698,12 @@
       </c>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Bloqueada</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>Pendente — o rascunho não aparece mais na lista da Nekt (arquivado ou excluído em 14–15/10)</t>
+          <t>Plano da conta inviabiliza rodar a conta (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="L4" s="7" t="inlineStr">
@@ -1719,7 +1713,7 @@
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>Conta sem fonte na Nekt hoje</t>
+          <t>Plano da conta inviabiliza rodar a conta (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="N4" s="7" t="inlineStr">
@@ -1745,14 +1739,10 @@
       </c>
       <c r="S4" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
-        </is>
-      </c>
-      <c r="T4" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>Depende de mudança de plano; sem previsão</t>
+        </is>
+      </c>
+      <c r="T4" s="7" t="n"/>
       <c r="U4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
@@ -1801,12 +1791,12 @@
       </c>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Não precisa manter (duplicidade)</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Pendente — o rascunho não aparece mais na lista da Nekt (arquivado ou excluído em 14–15/10)</t>
+          <t>Duplicidade informada pela Jussara em 16/10</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
@@ -1816,7 +1806,7 @@
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>Conta sem fonte na Nekt hoje</t>
+          <t>Duplicidade informada pela Jussara em 16/10</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
@@ -1846,14 +1836,10 @@
       </c>
       <c r="S5" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
-        </is>
-      </c>
-      <c r="T5" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>Não integrar a conta 2; decidir o destino da conta 1 (wypN, 0 linhas)</t>
+        </is>
+      </c>
+      <c r="T5" s="7" t="n"/>
       <c r="U5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
@@ -1902,12 +1888,12 @@
       </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Pendente — o rascunho não aparece mais na lista da Nekt (arquivado ou excluído em 14–15/10)</t>
+          <t>Inativo na agência (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="L6" s="7" t="inlineStr">
@@ -1917,7 +1903,7 @@
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
-          <t>Conta sem fonte na Nekt hoje</t>
+          <t>Inativo na agência (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="N6" s="7" t="inlineStr">
@@ -1931,14 +1917,10 @@
       <c r="R6" s="7" t="inlineStr"/>
       <c r="S6" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
-        </is>
-      </c>
-      <c r="T6" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>Não integrar; pedir desvínculo ou pausa no MCC</t>
+        </is>
+      </c>
+      <c r="T6" s="7" t="n"/>
       <c r="U6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
@@ -1987,12 +1969,12 @@
       </c>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>Pendente — o rascunho não aparece mais na lista da Nekt (arquivado ou excluído em 14–15/10)</t>
+          <t>Inativo na agência (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
@@ -2002,7 +1984,7 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Conta sem fonte na Nekt hoje</t>
+          <t>Inativo na agência (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
@@ -2016,14 +1998,10 @@
       <c r="R7" s="7" t="inlineStr"/>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
-        </is>
-      </c>
-      <c r="T7" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>Não integrar; pedir desvínculo ou pausa no MCC</t>
+        </is>
+      </c>
+      <c r="T7" s="7" t="n"/>
       <c r="U7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -2077,7 +2055,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>Pendente — rascunho criado, falta OAuth</t>
+          <t>Pendente — aguardando autorização (informado pela jussara em 16/10)</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr">
@@ -2087,7 +2065,7 @@
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>OAuth com usuário Google que administra o MCC</t>
+          <t>Aguardando autorização (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="N8" s="7" t="inlineStr">
@@ -2113,14 +2091,10 @@
       </c>
       <c r="S8" s="7" t="inlineStr">
         <is>
-          <t>Encaminhar link de autorização ao administrador do MCC</t>
-        </is>
-      </c>
-      <c r="T8" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>Aguardar a autorização do cliente/administrador; depois OAuth e publicar</t>
+        </is>
+      </c>
+      <c r="T8" s="7" t="n"/>
       <c r="U8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
@@ -2347,12 +2321,12 @@
       </c>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Não precisa manter (decisão: não conectar por ora)</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>Pendente — o rascunho não aparece mais na lista da Nekt (arquivado ou excluído em 14–15/10)</t>
+          <t>E-mail do João de 30/09: conta de backup não será conectada à Nekt por ora (Jussara respondeu "Ciente" em 01/10)</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
@@ -2362,7 +2336,7 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>Conta sem fonte na Nekt hoje</t>
+          <t>E-mail do João de 30/09: conta de backup não será conectada à Nekt por ora (Jussara respondeu "Ciente" em 01/10)</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
@@ -2388,7 +2362,7 @@
       </c>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>NÃO autorizar nem publicar até o João confirmar que o bloqueio estabilizou (e-mail de 30/09: conta de backup não será conectada à Nekt por enquanto)</t>
+          <t>Não conectar; rever se o João avisar que o bloqueio estabilizou</t>
         </is>
       </c>
       <c r="T11" s="7" t="n"/>
@@ -2449,7 +2423,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Pendente — o rascunho não aparece mais na lista da Nekt (arquivado ou excluído em 14–15/10)</t>
+          <t>Pendente — aguardando autorização (informado pela jussara em 16/10)</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">
@@ -2459,7 +2433,7 @@
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>Conta sem fonte na Nekt hoje</t>
+          <t>Aguardando autorização (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
@@ -2477,14 +2451,10 @@
       <c r="R12" s="7" t="inlineStr"/>
       <c r="S12" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
-        </is>
-      </c>
-      <c r="T12" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>Aguardar a autorização do cliente/administrador; depois OAuth e publicar</t>
+        </is>
+      </c>
+      <c r="T12" s="7" t="n"/>
       <c r="U12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
@@ -2533,12 +2503,12 @@
       </c>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>Pendente — o rascunho não aparece mais na lista da Nekt (arquivado ou excluído em 14–15/10)</t>
+          <t>Inativo na agência (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
@@ -2548,7 +2518,7 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Conta sem fonte na Nekt hoje</t>
+          <t>Inativo na agência (informado pela Jussara em 16/10)</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -2566,14 +2536,10 @@
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
-        </is>
-      </c>
-      <c r="T13" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>Não integrar; pedir desvínculo ou pausa no MCC</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="n"/>
       <c r="U13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
@@ -23286,7 +23252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23453,20 +23419,20 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Account Manager (confirmar se a conta ainda é cliente)</t>
+          <t>Account Manager / cliente (autorização)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth</t>
+          <t>Aguardar a autorização; depois OAuth e publicar</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>AÇO MANAUS; BRAGA MOTORS BMW; CDL MANAUS; DR. CABRAL (conta 2 NOVA); HOPE BAY PARK; JULIA HERRERA; SANTO REMÉDIO (conta viva); TUBOAÇOS DA AMAZÔNIA; UIARA AMAZON RESORT</t>
+          <t>AÇO MANAUS; BRAGA MOTORS BMW; PNEU FORTE VAREJO; TUBOAÇOS DA AMAZÔNIA</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -23493,7 +23459,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Encaminhar link de autorização ao administrador do MCC</t>
+          <t>Encerrar a AMd2 na interface depois de integrar a conta viva; histórico preservado</t>
         </is>
       </c>
       <c r="E6" s="7" t="n">
@@ -23501,12 +23467,12 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>PNEU FORTE VAREJO</t>
+          <t>SANTO REMÉDIO</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Bloqueada</t>
         </is>
       </c>
     </row>
@@ -23528,7 +23494,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Encerrar a AMd2 na interface depois de integrar a conta viva; histórico preservado</t>
+          <t>Duplicidade informada: não integrar a conta 2; decidir o destino da conta 1 (wypN)</t>
         </is>
       </c>
       <c r="E7" s="7" t="n">
@@ -23536,12 +23502,12 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>SANTO REMÉDIO</t>
+          <t>DR. CABRAL (conta 1)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Conectada</t>
         </is>
       </c>
     </row>
@@ -23563,7 +23529,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Integrar a conta NOVA e então decidir encerrar a wypN</t>
+          <t>Reautorizar a fonte OzfZ</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -23571,12 +23537,12 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>DR. CABRAL (conta 1)</t>
+          <t>PRESTEX</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Conectada</t>
+          <t>Bloqueada</t>
         </is>
       </c>
     </row>
@@ -23593,12 +23559,12 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
+          <t>João (confirmar ID) + Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Reautorizar a fonte OzfZ</t>
+          <t>Confirmar ID/vínculo da Braga Venda Direta no MCC; depois criar rascunho</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -23606,7 +23572,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>PRESTEX</t>
+          <t>BRAGA VENDA DIRETA</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -23633,7 +23599,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Confirmar ID/vínculo da Braga Venda Direta no MCC; depois criar rascunho</t>
+          <t>Confirmar ID/vínculo da Comac no MCC; depois criar rascunho</t>
         </is>
       </c>
       <c r="E10" s="7" t="n">
@@ -23641,7 +23607,7 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>BRAGA VENDA DIRETA</t>
+          <t>COMAC</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -23658,30 +23624,30 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Google Ads</t>
+          <t>Meta Ads</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>João (confirmar ID) + Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
+          <t>Admin do BM Meta + AM</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Confirmar ID/vínculo da Comac no MCC; depois criar rascunho</t>
+          <t>Decidir reativar ou encerrar a conta</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>COMAC</t>
+          <t>DR. CABRAL; MILLENIUM</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Conectada</t>
         </is>
       </c>
     </row>
@@ -23698,25 +23664,25 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Admin do BM Meta + AM</t>
+          <t>Jussara (OAuth) / admin do BM Meta</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Decidir reativar ou encerrar a conta</t>
+          <t>Abrir link de autorização, depois validar/criar camada/publicar</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>DR. CABRAL; MILLENIUM</t>
+          <t>CAA | MARCENARIA; DANIELE BARROCO; Health&amp;CO; Portal Vidros; RCB Imóveis; Rocha e Paiva; [LB - 28] - [02]</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Conectada</t>
+          <t>Pendente</t>
         </is>
       </c>
     </row>
@@ -23733,25 +23699,25 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Jussara (OAuth) / admin do BM Meta</t>
+          <t>Nekt (Jussara)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Abrir link de autorização, depois validar/criar camada/publicar</t>
+          <t>Conferir dado após a terça 20/10 e somar à Trusted</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>7</v>
+        <v>56</v>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>CAA | MARCENARIA; DANIELE BARROCO; Health&amp;CO; Portal Vidros; RCB Imóveis; Rocha e Paiva; [LB - 28] - [02]</t>
+          <t>ACESSO SAÚDE; AMAZONCOPY; AMZ GERADORES; ANIMATIV; ARENA TINTAS [E-COM + AQUISIÇÃO]; ARTRIN; BA ELÉTRICA; BEST CAR; BIGAZINE [E-COM + AQUISIÇÃO]; BRAGA (Grupo Completo); CAA ALUMÍNIO; CAA TINTAS; CDL MANAUS; COMAC; Consórcio Chevrolet; DEB TRANSPORTADORA; DON WATCHES; DR. CABRAL; HAGE; HOSPITAL SANTA JÚLIA; INFORCELL; Japurá Pneus; KIFFER; LEAP MOTORS; MILLENIUM; MOVE RENTAL CARS; Neo Vila Adrianopolis Empreendimento Ads; PMZ ESCOLA DE MECÂNICOS; PMZ GRUPO ECOMM; PNEU EXPRESS; PNEU FORTE DISTRIBUIDORA; PNEU FORTE VAREJO; Parque das Torres Ads; REI DAS MANGUEIRAS; RODRIX; Residencial Boa Vista Ads; SMILE PNEUS; STEEL PORT; THEREZINHA; Tropical Multiloja - Ativo; UNIPAR; VEGA Bajaj Manaus (AM) - Anúncios; VOIKÉ; Vanguarda Comunicação; Vbot</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Conectada</t>
         </is>
       </c>
     </row>
@@ -23763,30 +23729,30 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>RD Station</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Nekt (Jussara)</t>
+          <t>Analista Inbound (Bryan) + admin da conta RD do CDL</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Conferir dado após a terça 20/10 e somar à Trusted</t>
+          <t>Conferir plano/permissão da conta RD do CDL e reautorizar</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>ACESSO SAÚDE; AMAZONCOPY; AMZ GERADORES; ANIMATIV; ARENA TINTAS [E-COM + AQUISIÇÃO]; ARTRIN; BA ELÉTRICA; BEST CAR; BIGAZINE [E-COM + AQUISIÇÃO]; BRAGA (Grupo Completo); CAA ALUMÍNIO; CAA TINTAS; CDL MANAUS; COMAC; Consórcio Chevrolet; DEB TRANSPORTADORA; DON WATCHES; DR. CABRAL; HAGE; HOSPITAL SANTA JÚLIA; INFORCELL; Japurá Pneus; KIFFER; LEAP MOTORS; MILLENIUM; MOVE RENTAL CARS; Neo Vila Adrianopolis Empreendimento Ads; PMZ ESCOLA DE MECÂNICOS; PMZ GRUPO ECOMM; PNEU EXPRESS; PNEU FORTE DISTRIBUIDORA; PNEU FORTE VAREJO; Parque das Torres Ads; REI DAS MANGUEIRAS; RODRIX; Residencial Boa Vista Ads; SMILE PNEUS; STEEL PORT; THEREZINHA; Tropical Multiloja - Ativo; UNIPAR; VEGA Bajaj Manaus (AM) - Anúncios; VOIKÉ; Vanguarda Comunicação; Vbot</t>
+          <t>CDL</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Conectada</t>
+          <t>Bloqueada</t>
         </is>
       </c>
     </row>
@@ -23803,25 +23769,25 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound (Bryan) + admin da conta RD do CDL</t>
+          <t>Analista Inbound (Bryan) + admin da conta RD do cliente (a confirmar)</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Conferir plano/permissão da conta RD do CDL e reautorizar</t>
+          <t>Analista Inbound confirmar se a conta RD existe; se sim, recriar o rascunho</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>CDL</t>
+          <t>LEGACY PNEUS; LOVOL; TARGO CONSULTORIA</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Pendente</t>
         </is>
       </c>
     </row>
@@ -23838,20 +23804,20 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound (Bryan) + admin da conta RD do cliente (a confirmar)</t>
+          <t>Analista Inbound (Joyce) + admin da conta RD do cliente (a confirmar)</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound confirmar se a conta RD existe; se sim, recriar o rascunho</t>
+          <t>Encaminhar link de autorização ao administrador da conta RD</t>
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>LEGACY PNEUS; LOVOL; TARGO CONSULTORIA</t>
+          <t>BRAGA MOTOS - YAMAHA - VENDAS</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -23873,12 +23839,12 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound (Joyce) + admin da conta RD do cliente (a confirmar)</t>
+          <t>Analista Inbound (Juan Carlos) + admin da conta RD do cliente (a confirmar)</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Encaminhar link de autorização ao administrador da conta RD</t>
+          <t>Analista Inbound confirmar se a conta RD existe; se sim, recriar o rascunho</t>
         </is>
       </c>
       <c r="E17" s="7" t="n">
@@ -23886,7 +23852,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>BRAGA MOTOS - YAMAHA - VENDAS</t>
+          <t>BRAGA VEÍCULOS VENDAS - PÓS VENDA</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -23908,12 +23874,12 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound (Juan Carlos) + admin da conta RD do cliente (a confirmar)</t>
+          <t>Jussara (diagnóstico na Nekt) + Analista Inbound (Joyce)</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Analista Inbound confirmar se a conta RD existe; se sim, recriar o rascunho</t>
+          <t>Conferir se a conta RD do cliente tem contatos/conversões e a permissão da API</t>
         </is>
       </c>
       <c r="E18" s="7" t="n">
@@ -23921,12 +23887,12 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>BRAGA VEÍCULOS VENDAS - PÓS VENDA</t>
+          <t>AMZ IMPORTS</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Conectada</t>
         </is>
       </c>
     </row>
@@ -23943,20 +23909,20 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Jussara (diagnóstico na Nekt) + Analista Inbound (Joyce)</t>
+          <t>Nekt (Jussara)</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Conferir se a conta RD do cliente tem contatos/conversões e a permissão da API</t>
+          <t>Conferir carga e somar às Trusted de RD</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>AMZ IMPORTS</t>
+          <t>ARENA TINTAS; BAJAJ; BAP; BRAGA MOTOS - YAMAHA - PÓS VENDAS; BRAGA VEÍCULOS - VENDA DIRETA; BRAGA VEÍCULOS VAREJO; CAA ALUMÍNIO; CAA TINTAS; CHARÃO; CONSTROI INCORPORADORA; DISTRIBUIDORA PNEU FORTE; DOCTOR MAIS SAÚDE; HAGE ALIMENTOS; PMZ ESCOLA; RODRIX; ROYAL ENFIELD; SANTO REMÉDIO; SHIZEN; UNIPAR</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -23968,30 +23934,30 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>RD Station</t>
+          <t>Google Ads</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Nekt (Jussara)</t>
+          <t>Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Conferir carga e somar às Trusted de RD</t>
+          <t>Reautorizar no prazo da Google (23/10)</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>ARENA TINTAS; BAJAJ; BAP; BRAGA MOTOS - YAMAHA - PÓS VENDAS; BRAGA VEÍCULOS - VENDA DIRETA; BRAGA VEÍCULOS VAREJO; CAA ALUMÍNIO; CAA TINTAS; CHARÃO; CONSTROI INCORPORADORA; DISTRIBUIDORA PNEU FORTE; DOCTOR MAIS SAÚDE; HAGE ALIMENTOS; PMZ ESCOLA; RODRIX; ROYAL ENFIELD; SANTO REMÉDIO; SHIZEN; UNIPAR</t>
+          <t>ACESSO SAÚDE; AMAZONCOPY; AMZ GERADORES; ARENA TINTAS; BA ELÉTRICA; BIGAZINE; CAA ALUMÍNIO; CAA TINTAS; COLMEIA; CONSTRÓI INCORPORADORA; DEB TRANSPORTADORA; DOCTOR MAIS; DON WATCHES (conta 2); HOSPITAL SANTA JÚLIA; MILLENIUM; MOVE RENTAL CARS; PMZ ESCOLA DE MECÂNICOS; PMZ GRUPO ECOMM; PMZ GRUPO LOJA; PNEU EXPRESS; PNEU FORTE DISTRIBUIDORA; REI DAS MANGUEIRAS; RODRIX; SMILE PNEUS; STEEL PORT</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -24013,60 +23979,60 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
+          <t>Jussara + administrador do MCC</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Reautorizar no prazo da Google (23/10)</t>
+          <t>Não integrar; solicitar desvínculo da conta do MCC</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>ACESSO SAÚDE; AMAZONCOPY; AMZ GERADORES; ARENA TINTAS; BA ELÉTRICA; BIGAZINE; CAA ALUMÍNIO; CAA TINTAS; COLMEIA; CONSTRÓI INCORPORADORA; DEB TRANSPORTADORA; DOCTOR MAIS; DON WATCHES (conta 2); HOSPITAL SANTA JÚLIA; MILLENIUM; MOVE RENTAL CARS; PMZ ESCOLA DE MECÂNICOS; PMZ GRUPO ECOMM; PMZ GRUPO LOJA; PNEU EXPRESS; PNEU FORTE DISTRIBUIDORA; REI DAS MANGUEIRAS; RODRIX; SMILE PNEUS; STEEL PORT</t>
+          <t>LOJA | NOVA ERA BV | PIX; LOJA | NOVA ERA PVH | PIX; NOVA ERA MAO | LOJAS; NOVA ERA | MANAUS | ECOMM; NOVA ERA | PORTO VELHO | ECOMM</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Conectada</t>
+          <t>Fora do escopo (Nova Era)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Google Ads</t>
+          <t>LinkedIn Ads</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Jussara + administrador do MCC</t>
+          <t>Analista da conta</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Não integrar; solicitar desvínculo da conta do MCC</t>
+          <t>Levantar ID da conta e decidir se entra no escopo</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>LOJA | NOVA ERA BV | PIX; LOJA | NOVA ERA PVH | PIX; NOVA ERA MAO | LOJAS; NOVA ERA | MANAUS | ECOMM; NOVA ERA | PORTO VELHO | ECOMM</t>
+          <t>ALMEIDA E BARRETO; AMAZONCOPY; PRESTEX; TUBOAÇOS</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Fora do escopo (Nova Era)</t>
+          <t>Sem conexão</t>
         </is>
       </c>
     </row>
@@ -24078,7 +24044,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>LinkedIn Ads</t>
+          <t>TikTok Ads</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -24092,49 +24058,14 @@
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>ALMEIDA E BARRETO; AMAZONCOPY; PRESTEX; TUBOAÇOS</t>
+          <t>BA ELÉTRICA; SANTO REMÉDIO; TUBOAÇOS</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>Sem conexão</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>TikTok Ads</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Analista da conta</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>Levantar ID da conta e decidir se entra no escopo</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>BA ELÉTRICA; SANTO REMÉDIO; TUBOAÇOS</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>Sem conexão</t>
         </is>
@@ -24208,11 +24139,11 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Reautorizar no prazo da Google (23/10) (25); Encaminhar link de autorização ao administrador do MCC (1); Reautorizar a fonte OzfZ (1); Encerrar a AMd2 na interface depois de integrar a conta viva; histórico preservado (1); Integrar a conta NOVA e então decidir encerrar a wypN (1)</t>
+          <t>Reautorizar no prazo da Google (23/10) (25); Reautorizar a fonte OzfZ (1); Encerrar a AMd2 na interface; histórico preservado (1); Duplicidade do Dr. Cabral conta 2: decidir o destino da conta 1 (1)</t>
         </is>
       </c>
       <c r="D2" s="7" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
@@ -24288,7 +24219,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Account Manager (confirmar se a conta ainda é cliente)</t>
+          <t>Account Manager / cliente (autorização)</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -24298,11 +24229,11 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Confirmar com o AM se a conta ainda é cliente; se sim, recriar o rascunho e pedir o OAuth (9)</t>
+          <t>Aguardar a autorização; depois OAuth e publicar (4)</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
@@ -24384,11 +24315,11 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Não integrar; solicitar desvínculo da conta do MCC (5)</t>
+          <t>Não integrar; solicitar desvínculo ou pausa no MCC: 5 Nova Era, 2 Pátio Gourmet, 1 Olá Casa Nova, Hope Bay Park, Julia Herrera, UIARA (11)</t>
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
@@ -24704,7 +24635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -24871,6 +24802,13 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>• ATUALIZAÇÃO DE 16/10 (fim da tarde), status das 10 contas Google pendentes informado pela Jussara: AGUARDANDO AUTORIZAÇÃO — Aço Manaus, Braga Motors BMW, Pneu Forte Varejo, Tuboaços; BLOQUEADA POR PLANO — CDL Manaus; DUPLICIDADE — Dr. Cabral conta 2; INATIVOS NA AGÊNCIA — Hope Bay Park, Julia Herrera, UIARA; DECISÃO POR E-MAIL — Santo Remédio conta viva (não conectar por ora, e-mail do João de 30/09). Os cinco últimos saem das contas aplicáveis. Hope Bay, Julia e UIARA continuam no MCC e gastando (R$ 14.688,85 em 13/09–12/10).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Planilha oficial #1743: revisão de textos, Cronograma e Pendências alinhados às categorias
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNtRG1wGaTmzdzTc1r8f3Q
</commit_message>
<xml_diff>
--- a/docs/nekt/inventario-contas-1743-2026-10-16.xlsx
+++ b/docs/nekt/inventario-contas-1743-2026-10-16.xlsx
@@ -541,7 +541,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Posição de 16/10/2026: status de integração relido na Nekt pela varredura da manhã (252 fontes publicadas). Substitui as versões de 13/10 e 15/10, que ficam só como histórico. Gasto: Meta 7 dias (02 a 08/10), Google 30 dias (até 05/10).</t>
+          <t>Posição de 16/10/2026 (noite): status de integração relido na Nekt pela varredura da manhã (252 fontes publicadas) e ajustado pelas informações da Jussara durante o dia (ex-clientes, duplicidade, decisões). Substitui as versões de 13/10 e 15/10, que ficam só como histórico. Gasto: Meta 7 dias (02 a 08/10), Google 30 dias (13/09 a 12/10).</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
@@ -836,7 +835,7 @@
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• Google Ads: 40 contas conectadas (a Olá Casa Nova saiu: ex-cliente). As 14 que falharam por cota 429 em 14/10 voltaram a ter sucesso em 16/10, e a Prestex (OzfZ) também (dado até 12/10, ainda fora da Trusted). 10 pendentes (as 2 contas Pátio Gourmet saíram: ex-cliente): os rascunhos de 05/10 foram removidos da lista da Nekt (só o H3hJ restou), então precisam de confirmação de que a conta ainda é cliente. 3 bloqueadas: Santo Remédio (AMd2, conta saiu do MCC), Comac e Braga Venda Direta (IDs que não aparecem no MCC). Santo Remédio (513-801-6841): o e-mail do João de 30/09 diz para não conectar a conta de backup por ora; não autorizar sem confirmação.</t>
+          <t>• Google Ads: 41 contas conectadas (inclui a Prestex, OzfZ, com sucesso em 16/10, dado semanal até 12/10, ainda fora da Trusted, e a Dmello, URNQ). As 14 que falharam por cota 429 em 14/10 voltaram a ter sucesso em 16/10. 5 pendentes: 4 aguardando autorização (Aço Manaus, Braga Motors BMW, Pneu Forte Varejo, Tuboaços) e a conta própria da Vanguarda (750-265-3880, decidir se entra). 4 bloqueadas: CDL Manaus (o plano da conta inviabiliza rodar, sem previsão), Santo Remédio AMd2 (conta saiu do MCC), Comac e Braga Venda Direta (IDs que não aparecem no MCC). 8 fora do que precisa manter: Pátio Gourmet ×2, Olá Casa Nova, Hope Bay Park, Julia Herrera e UIARA (ex-clientes/inativos), Dr. Cabral conta 2 (duplicidade; qual das duas é a duplicada foi presumido) e Santo Remédio conta viva (e-mail do João de 30/09: não conectar por ora). 5 Nova Era fora do escopo.</t>
         </is>
       </c>
     </row>
@@ -885,7 +884,7 @@
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>1) Administrador do MCC Google Ads (1704439246): confirmar quais contas dos 12 pendentes ainda são clientes e autorizar o OAuth das que ficam; reautorizar o conector v2.53 (23/10); desvincular Nova Era. Responsável proposto: João Araújo (ADMIN do MCC, ver Premissas) — a confirmar.</t>
+          <t>1) Administrador do MCC Google Ads (1704439246): autorizar o OAuth das 4 contas que aguardam autorização; reautorizar o conector v2.53 das 41 contas conectadas (23/10); desvincular ou pausar as 11 contas de ex-clientes/inativos que seguem no MCC e gastando (Nova Era ×5, UIARA, Pátio Gourmet ×2, Olá Casa Nova, Hope Bay, Julia Herrera: R$ 46.430,03 em 13/09–12/10); decidir a conta própria da Vanguarda. Responsável proposto: João Araújo (ADMIN do MCC, ver Premissas) — a confirmar.</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1317,6 @@
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -23252,7 +23250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23459,7 +23457,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Encerrar a AMd2 na interface depois de integrar a conta viva; histórico preservado</t>
+          <t>Encerrar a AMd2 na interface (a conta saiu do MCC; histórico preservado). A conta viva (513-801-6841) não será conectada por ora: e-mail do João de 30/09</t>
         </is>
       </c>
       <c r="E6" s="7" t="n">
@@ -23529,7 +23527,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Reautorizar a fonte OzfZ</t>
+          <t>Conferida em 16/10: sucesso, dado semanal até 12/10, leitura bate com o MCC. Decidir se entra na união da Trusted (granularidade semanal); reautorização v2.53 incluída na linha de 23/10</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -23542,7 +23540,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Conectada</t>
         </is>
       </c>
     </row>
@@ -23953,11 +23951,11 @@
         </is>
       </c>
       <c r="E20" s="7" t="n">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>ACESSO SAÚDE; AMAZONCOPY; AMZ GERADORES; ARENA TINTAS; BA ELÉTRICA; BIGAZINE; CAA ALUMÍNIO; CAA TINTAS; COLMEIA; CONSTRÓI INCORPORADORA; DEB TRANSPORTADORA; DOCTOR MAIS; DON WATCHES (conta 2); HOSPITAL SANTA JÚLIA; MILLENIUM; MOVE RENTAL CARS; PMZ ESCOLA DE MECÂNICOS; PMZ GRUPO ECOMM; PMZ GRUPO LOJA; PNEU EXPRESS; PNEU FORTE DISTRIBUIDORA; REI DAS MANGUEIRAS; RODRIX; SMILE PNEUS; STEEL PORT</t>
+          <t>As 41 contas Google Ads conectadas (fontes publicadas ativas; lista completa na aba Contas, categoria Conectada)</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -24068,6 +24066,111 @@
       <c r="G23" s="7" t="inlineStr">
         <is>
           <t>Sem conexão</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Account Manager (Betina Gava, analista) / admin do MCC (a confirmar)</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>CDL Manaus: o plano da conta inviabiliza rodar; depende de mudança de plano, sem previsão</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>CDL MANAUS (google-ads-zksL, rascunho)</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Bloqueada</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Decidir se a conta própria da Vanguarda (750-265-3880) entra; se sim, criar o rascunho e pedir o OAuth</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>VANGUARDA COMUNICAÇÃO (conta própria)</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Jussara + administrador do MCC</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Não integrar; solicitar desvínculo ou pausa no MCC (ex-clientes/inativos)</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>UIARA; PÁTIO GOURMET (2 contas); OLÁ CASA NOVA; HOPE BAY PARK; JULIA HERRERA</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Não precisa manter (ex-cliente)</t>
         </is>
       </c>
     </row>
@@ -24083,7 +24186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -24139,11 +24242,11 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Reautorizar no prazo da Google (23/10) (25); Reautorizar a fonte OzfZ (1); Encerrar a AMd2 na interface; histórico preservado (1); Duplicidade do Dr. Cabral conta 2: decidir o destino da conta 1 (1)</t>
+          <t>Reautorizar o conector v2.53 no prazo da Google (23/10) (41, inclui a Prestex); Encerrar a AMd2 na interface; histórico preservado (1); Duplicidade do Dr. Cabral conta 2: decidir o destino da conta 1 (1)</t>
         </is>
       </c>
       <c r="D2" s="7" t="n">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
@@ -24619,6 +24722,66 @@
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>docs/nekt/solicitacoes-1743-2026-10-15.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Account Manager / analista do CDL Manaus (Betina Gava) + admin do MCC (a confirmar)</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>E-mail + tarefa no VJOB</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>CDL Manaus: o plano da conta inviabiliza rodar; depende de mudança de plano, sem previsão (1)</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>docs/nekt/solicitacoes-1743-2026-10-15.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Administrador do MCC Google Ads 170-443-9246 (a confirmar)</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>E-mail + tarefa no VJOB</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Decidir se a conta própria da Vanguarda (750-265-3880) entra; se sim, criar o rascunho e pedir o OAuth (1)</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>docs/nekt/solicitacoes-1743-2026-10-15.md</t>
         </is>
@@ -24635,7 +24798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -24809,6 +24972,13 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>• ATUALIZAÇÃO DE 16/10 (noite), revisão geral da planilha: textos do Resumo e do Cronograma alinhados às categorias da aba Contas (Google: 41 conectadas, 5 pendentes, 4 bloqueadas, 5 Nova Era, 8 fora do que precisa manter = 63 linhas); reautorização v2.53 passa a cobrir as 41 conectadas; Prestex marcada como conectada no Cronograma; adicionadas linhas para CDL, conta própria da Vanguarda e as 6 contas de ex-clientes/inativos que seguem no MCC. PREMISSAS MINHAS, a confirmar: CDL foi classificada como bloqueada (por plano); Dr. Cabral conta 2 (4YJU, 251-691-8741) foi presumida como a duplicada; AMd2 e as Meta f6h8/geQA (Santo Remédio) não foram abordadas pela Jussara e ficam como estavam; as datas continuam proposta.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>